<commit_message>
Apply conditional formatting to status flags on reconciliation sheet
</commit_message>
<xml_diff>
--- a/investment_reconciliation_tracker.xlsx
+++ b/investment_reconciliation_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gaspar\Data\Portfolio\investment-reconciliation-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50008239-5DB6-4F1A-AD56-D6A26A6F2D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89227116-B3CF-4F81-A60F-54F77F86832E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19296" yWindow="-96" windowWidth="19392" windowHeight="10536" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,15 +210,104 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -277,17 +366,17 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{27DF082A-EB9F-48D9-B5FC-859B5DFB74AB}" name="Reconciliation" displayName="Reconciliation" ref="A1:K11" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:K11" xr:uid="{27DF082A-EB9F-48D9-B5FC-859B5DFB74AB}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{DABA9359-B81E-4CC7-9CD0-11A733321E9E}" uniqueName="1" name="Fund ID" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{84A93B77-8E17-436F-B764-FA6B8C0BCF33}" uniqueName="2" name="Fund Name" queryTableFieldId="2" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{0AA2ADD2-1F88-421C-96A4-AFBC6806EDAB}" uniqueName="3" name="Asset Class" queryTableFieldId="3" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{DABA9359-B81E-4CC7-9CD0-11A733321E9E}" uniqueName="1" name="Fund ID" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{84A93B77-8E17-436F-B764-FA6B8C0BCF33}" uniqueName="2" name="Fund Name" queryTableFieldId="2" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{0AA2ADD2-1F88-421C-96A4-AFBC6806EDAB}" uniqueName="3" name="Asset Class" queryTableFieldId="3" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{549656F2-A49C-4EF6-9694-4013B6474E52}" uniqueName="4" name="Custodian Market Value" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{D075F688-B784-4AA8-A1A7-EBF09B5DC8B5}" uniqueName="5" name="Custodian Report Date" queryTableFieldId="5" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{D075F688-B784-4AA8-A1A7-EBF09B5DC8B5}" uniqueName="5" name="Custodian Report Date" queryTableFieldId="5" dataDxfId="12"/>
     <tableColumn id="6" xr3:uid="{4CF9E3C1-2B58-4DB0-AD49-BA2BEC81EAA2}" uniqueName="6" name="Statement Market Value" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{D1A427B3-AB28-4F86-8C5C-B32B8A9297D4}" uniqueName="7" name="Statememnt Report Date" queryTableFieldId="7" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{D1A427B3-AB28-4F86-8C5C-B32B8A9297D4}" uniqueName="7" name="Statememnt Report Date" queryTableFieldId="7" dataDxfId="11"/>
     <tableColumn id="8" xr3:uid="{8D0A0179-A009-4CF9-A491-2AFE4A9B0A23}" uniqueName="8" name="Difference ($)" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{BF7B0515-D1B8-49EF-81F9-65774A212195}" uniqueName="9" name="Difference (%)" queryTableFieldId="9"/>
-    <tableColumn id="10" xr3:uid="{1BC99722-B6B6-44CE-8650-1AFF082F56EA}" uniqueName="10" name="Status Flag" queryTableFieldId="10" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{EC8900C0-F1BD-466B-9A2F-8A2A27D1E372}" uniqueName="11" name="Issue Type" queryTableFieldId="11" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{1BC99722-B6B6-44CE-8650-1AFF082F56EA}" uniqueName="10" name="Status Flag" queryTableFieldId="10" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{EC8900C0-F1BD-466B-9A2F-8A2A27D1E372}" uniqueName="11" name="Issue Type" queryTableFieldId="11" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -608,25 +697,25 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2">
         <v>5200000</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45382</v>
       </c>
       <c r="F2">
         <v>5200000</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45382</v>
       </c>
       <c r="H2">
@@ -635,33 +724,33 @@
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
       <c r="D3">
         <v>12750000</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45382</v>
       </c>
       <c r="F3">
         <v>12900000</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45382</v>
       </c>
       <c r="H3">
@@ -670,33 +759,33 @@
       <c r="I3">
         <v>1.1764705882352941E-2</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
       <c r="D4">
         <v>3100000</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45382</v>
       </c>
       <c r="F4">
         <v>3100000</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45382</v>
       </c>
       <c r="H4">
@@ -705,33 +794,33 @@
       <c r="I4">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
         <v>8400000</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45382</v>
       </c>
       <c r="F5">
         <v>8400000</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45382</v>
       </c>
       <c r="H5">
@@ -740,33 +829,33 @@
       <c r="I5">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>29</v>
       </c>
       <c r="D6">
         <v>6600000</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45382</v>
       </c>
       <c r="F6">
         <v>6600000</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45351</v>
       </c>
       <c r="H6">
@@ -775,33 +864,33 @@
       <c r="I6">
         <v>0</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>18</v>
       </c>
       <c r="D7">
         <v>9800000</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45382</v>
       </c>
       <c r="F7">
         <v>9800000</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="1">
         <v>45382</v>
       </c>
       <c r="H7">
@@ -810,59 +899,59 @@
       <c r="I7">
         <v>0</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>23</v>
       </c>
       <c r="D8">
         <v>4250000</v>
       </c>
-      <c r="E8" s="2">
-        <v>45382</v>
-      </c>
-      <c r="G8" s="2">
-        <v>45382</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="E8" s="1">
+        <v>45382</v>
+      </c>
+      <c r="G8" s="1">
+        <v>45382</v>
+      </c>
+      <c r="J8" t="s">
         <v>36</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>18</v>
       </c>
       <c r="D9">
         <v>2100000</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45382</v>
       </c>
       <c r="F9">
         <v>2100000</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="1">
         <v>45382</v>
       </c>
       <c r="H9">
@@ -871,33 +960,33 @@
       <c r="I9">
         <v>0</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>26</v>
       </c>
       <c r="D10">
         <v>3750000</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45382</v>
       </c>
       <c r="F10">
         <v>3712500</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45382</v>
       </c>
       <c r="H10">
@@ -906,33 +995,33 @@
       <c r="I10">
         <v>0.01</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>29</v>
       </c>
       <c r="D11">
         <v>7300000</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>45382</v>
       </c>
       <c r="F11">
         <v>7300000</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>45382</v>
       </c>
       <c r="H11">
@@ -941,14 +1030,25 @@
       <c r="I11">
         <v>0</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" t="s">
         <v>14</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="STALE DATE">
+      <formula>NOT(ISERROR(SEARCH("STALE DATE",J1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="MISSING DATA">
+      <formula>NOT(ISERROR(SEARCH("MISSING DATA",J1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="BREAK">
+      <formula>NOT(ISERROR(SEARCH("BREAK",J1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>